<commit_message>
Update category column handling in dataset loading and instance creation
</commit_message>
<xml_diff>
--- a/Data/Datasets/Output/meta_feature_training_stats_.xlsx
+++ b/Data/Datasets/Output/meta_feature_training_stats_.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/38498c2a7fab902e/tuks/master/code/Thesis/Data/Datasets/Output/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/38498c2a7fab902e/tuks/master/code/Laptop/Data/Datasets/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="173" documentId="11_F25DC773A252ABDACC1048A2915872405ADE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF60EAB1-CDB3-450E-AB17-AE7C82F601B0}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="11_F25DC773A252ABDACC1048A2915872405ADE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750D6146-BAE7-49C0-87BF-7D43537F1862}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -151,7 +151,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +163,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -255,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -282,6 +297,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -980,7 +998,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37982CAE-0D25-43BC-94BB-81C8EE4EF796}">
-  <dimension ref="B2:I16"/>
+  <dimension ref="B2:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
@@ -1140,28 +1158,28 @@
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="13">
         <v>5.8151260504201598</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="14">
         <v>1</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="13">
         <v>0.84033613445378097</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="14">
         <v>64</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="13">
         <v>53.781512605042003</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="14">
         <v>136</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="13">
         <f>H8/255*100</f>
         <v>53.333333333333336</v>
       </c>
@@ -1194,28 +1212,28 @@
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="13">
         <v>5.3176470588235203</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="14">
         <v>2</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="13">
         <v>0.78431372549019596</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="14">
         <v>63</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="13">
         <v>24.705882352941099</v>
       </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4">
+      <c r="H10" s="14">
+        <v>0</v>
+      </c>
+      <c r="I10" s="13">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1248,36 +1266,30 @@
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="13">
         <v>4.9215686274509798</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="14">
         <v>34</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="13">
         <v>13.3333333333333</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="14">
         <v>115</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="13">
         <v>45.0980392156862</v>
       </c>
-      <c r="H12" s="1">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4">
+      <c r="H12" s="14">
+        <v>0</v>
+      </c>
+      <c r="I12" s="13">
         <f t="shared" si="1"/>
         <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E16">
-        <f>255-136</f>
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1289,5 +1301,6 @@
     <mergeCell ref="F2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>